<commit_message>
Recheck NPL_1 coding with stakeholder analysis
Recode after analyzing interviewee identity as federal governmental actor
(Department of Environment). Add Stakeholder Analysis sheet, correct several
codes (Problem_import, Problem_awareness_pol, Pol_tax, Sol_ban, Sol_segregation,
Sol_tax), and document RSCT note ambiguity.

Co-authored-by: Vaibhav <shivrain@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/interview_coding_NPL_1.xlsx
+++ b/interview_coding_NPL_1.xlsx
@@ -10,6 +10,7 @@
     <sheet name="Interview Coding" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Wide Format" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="Codebook Reference" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Stakeholder Analysis" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -539,7 +540,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Interview: NPL_1  |  Country: NEPAL  |  Actor: Environmental Department  |  Source: Interview Guideline — Environmental Department (June 2023)</t>
+          <t>Interview: NPL_1  |  Country: NEPAL  |  Actor: Federal governmental (Department of Environment / Ministry)  |  Source: Interview Guideline — Environmental Department (June 2023)</t>
         </is>
       </c>
     </row>
@@ -637,7 +638,7 @@
       </c>
       <c r="D8" s="5" t="inlineStr">
         <is>
-          <t>Environmental Department / Ministry of Forests and Environment respondent.</t>
+          <t>Federal governmental actor (Department of Environment). Uses first-person 'we' for policy implementation, ministry-only questions (4.a/4.b), and describes Chief Secretary committee oversight.</t>
         </is>
       </c>
     </row>
@@ -671,7 +672,7 @@
       </c>
       <c r="B10" s="5" t="inlineStr">
         <is>
-          <t>NA</t>
+          <t>low</t>
         </is>
       </c>
       <c r="C10" s="5" t="inlineStr">
@@ -679,7 +680,11 @@
           <t>high, medium, low, NA — lack of awareness among policy makers mentioned</t>
         </is>
       </c>
-      <c r="D10" s="5" t="inlineStr"/>
+      <c r="D10" s="5" t="inlineStr">
+        <is>
+          <t>Low political priority among decision-makers: 'no political will', plastics/waste 'not a priority' and 'stops at major' level.</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="4" t="inlineStr">
@@ -721,7 +726,7 @@
       </c>
       <c r="D12" s="5" t="inlineStr">
         <is>
-          <t>Blocking sewer systems; leakage into waterways.</t>
+          <t>Blocking sewer systems; leakage into waterways; landfill pressure.</t>
         </is>
       </c>
     </row>
@@ -765,7 +770,7 @@
       </c>
       <c r="D14" s="5" t="inlineStr">
         <is>
-          <t>Inadequate waste management; recycling participation via MRFs discussed.</t>
+          <t>Inadequate waste management; limited economically viable recycling for single-use items.</t>
         </is>
       </c>
     </row>
@@ -861,7 +866,7 @@
       </c>
       <c r="B19" s="4" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>yes</t>
         </is>
       </c>
       <c r="C19" s="4" t="inlineStr">
@@ -869,7 +874,11 @@
           <t>Plastic imports are a problem; was mentioned: yes/no</t>
         </is>
       </c>
-      <c r="D19" s="4" t="inlineStr"/>
+      <c r="D19" s="4" t="inlineStr">
+        <is>
+          <t>Import is part of the problem space: ban on production, import, and use of bags under 40 microns explicitly targets imported plastics.</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="5" t="inlineStr">
@@ -889,7 +898,7 @@
       </c>
       <c r="D20" s="5" t="inlineStr">
         <is>
-          <t>Waterways, urban systems, forests, health (burning/indoor), agriculture gaps in Chitwan.</t>
+          <t>Water (rivers/lakes), cities (sewers/urban), biodiversity (forests), health (burning/indoor air), agriculture (research gap noted for Chitwan).</t>
         </is>
       </c>
     </row>
@@ -969,7 +978,7 @@
       </c>
       <c r="D24" s="5" t="inlineStr">
         <is>
-          <t>Multi-level governance (national, district, municipal) with implementation gaps.</t>
+          <t>Challenges differ across national, district, and municipal levels; SWM Act revision needed for federal governance alignment.</t>
         </is>
       </c>
     </row>
@@ -1027,7 +1036,7 @@
       </c>
       <c r="D27" s="4" t="inlineStr">
         <is>
-          <t>Department of Environment, Chief Secretary committee, Commerce and Supplies.</t>
+          <t>Department of Environment, Chief Secretary committee, Department of Commerce and Supplies.</t>
         </is>
       </c>
     </row>
@@ -1067,7 +1076,7 @@
       </c>
       <c r="D29" s="4" t="inlineStr">
         <is>
-          <t>Local governments lead waste management.</t>
+          <t>Local governments lead waste management and collection.</t>
         </is>
       </c>
     </row>
@@ -1151,7 +1160,7 @@
       </c>
       <c r="D33" s="4" t="inlineStr">
         <is>
-          <t>Not much research on plastic effects; more research needed.</t>
+          <t>Cites studies on microplastics; notes limited research on health/environmental effects.</t>
         </is>
       </c>
     </row>
@@ -1173,7 +1182,7 @@
       </c>
       <c r="D34" s="5" t="inlineStr">
         <is>
-          <t>Household waste collection with 300 NPR/month incentive for reduction.</t>
+          <t>Household waste reduction discussed; 300 NPR/month collector incentive mentioned (household incentive, not a product tax).</t>
         </is>
       </c>
     </row>
@@ -1213,7 +1222,7 @@
       </c>
       <c r="D36" s="5" t="inlineStr">
         <is>
-          <t>Private contractors and market monitoring.</t>
+          <t>Private contractors, plastic producers, and markets monitored by Department of Environment.</t>
         </is>
       </c>
     </row>
@@ -1275,7 +1284,7 @@
       </c>
       <c r="D39" s="4" t="inlineStr">
         <is>
-          <t>Funds exist but are not released; earmarked funds may be frozen.</t>
+          <t>Funds exist but are not released; earmarked funds may be frozen if unused.</t>
         </is>
       </c>
     </row>
@@ -1317,7 +1326,11 @@
           <t>Lack of infrastructure</t>
         </is>
       </c>
-      <c r="D41" s="4" t="inlineStr"/>
+      <c r="D41" s="4" t="inlineStr">
+        <is>
+          <t>Facilities exist in at least some contexts ('facility is there'); not coded as a primary lack-of-infrastructure barrier.</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="5" t="inlineStr">
@@ -1417,7 +1430,7 @@
       </c>
       <c r="D46" s="5" t="inlineStr">
         <is>
-          <t>Documentaries, traditional/social media, website materials.</t>
+          <t>Government documentaries, traditional/social media, website materials.</t>
         </is>
       </c>
     </row>
@@ -1483,7 +1496,7 @@
       </c>
       <c r="B50" s="5" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>no</t>
         </is>
       </c>
       <c r="C50" s="5" t="inlineStr">
@@ -1493,7 +1506,7 @@
       </c>
       <c r="D50" s="5" t="inlineStr">
         <is>
-          <t>300 NPR/month incentive for households reducing waste.</t>
+          <t>No levy/tax on specific products coded. The 300 NPR/month measure is a household waste-reduction incentive for collectors, not a bag tax/levy.</t>
         </is>
       </c>
     </row>
@@ -1537,7 +1550,7 @@
       </c>
       <c r="D52" s="5" t="inlineStr">
         <is>
-          <t>Biodegradable starch bags discussed as existing alternative.</t>
+          <t>Biodegradable starch bags discussed as existing but costly alternative.</t>
         </is>
       </c>
     </row>
@@ -1595,7 +1608,7 @@
       </c>
       <c r="D55" s="4" t="inlineStr">
         <is>
-          <t>Material recovery facilities and recycling to processing units.</t>
+          <t>Material recovery facilities send recyclables to processing units.</t>
         </is>
       </c>
     </row>
@@ -1655,7 +1668,11 @@
           <t>Procedural measures to establish lead agency</t>
         </is>
       </c>
-      <c r="D58" s="5" t="inlineStr"/>
+      <c r="D58" s="5" t="inlineStr">
+        <is>
+          <t>High-level committee chaired by Chief Secretary oversees measures.</t>
+        </is>
+      </c>
     </row>
     <row r="59">
       <c r="A59" s="4" t="inlineStr">
@@ -1673,7 +1690,11 @@
           <t>Clear responsibilities</t>
         </is>
       </c>
-      <c r="D59" s="4" t="inlineStr"/>
+      <c r="D59" s="4" t="inlineStr">
+        <is>
+          <t>EPR framed as key missing responsibility mechanism.</t>
+        </is>
+      </c>
     </row>
     <row r="60">
       <c r="A60" s="5" t="inlineStr">
@@ -1727,7 +1748,7 @@
       </c>
       <c r="B62" s="5" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>no</t>
         </is>
       </c>
       <c r="C62" s="5" t="inlineStr">
@@ -1735,7 +1756,11 @@
           <t>Segregation of waste</t>
         </is>
       </c>
-      <c r="D62" s="5" t="inlineStr"/>
+      <c r="D62" s="5" t="inlineStr">
+        <is>
+          <t>Collection/recycling encouraged, but segregation not proposed as a forward solution.</t>
+        </is>
+      </c>
     </row>
     <row r="63">
       <c r="A63" s="4" t="inlineStr">
@@ -1839,7 +1864,7 @@
       </c>
       <c r="B68" s="5" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>no</t>
         </is>
       </c>
       <c r="C68" s="5" t="inlineStr">
@@ -1857,7 +1882,7 @@
       </c>
       <c r="B69" s="4" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>no</t>
         </is>
       </c>
       <c r="C69" s="4" t="inlineStr">
@@ -1865,7 +1890,11 @@
           <t>Ban of products</t>
         </is>
       </c>
-      <c r="D69" s="4" t="inlineStr"/>
+      <c r="D69" s="4" t="inlineStr">
+        <is>
+          <t>Bans described as existing policy; forward-looking solutions emphasize EPR, R&amp;D, communication, and mitigation/adaptation rather than new bans.</t>
+        </is>
+      </c>
     </row>
     <row r="70">
       <c r="A70" s="5" t="inlineStr">
@@ -1885,7 +1914,7 @@
       </c>
       <c r="D70" s="5" t="inlineStr">
         <is>
-          <t>Financial support identified in Q10 follow-up.</t>
+          <t>Financial support identified in Q10.</t>
         </is>
       </c>
     </row>
@@ -1907,7 +1936,7 @@
       </c>
       <c r="D71" s="4" t="inlineStr">
         <is>
-          <t>Infrastructural support identified in Q10 follow-up.</t>
+          <t>Infrastructural support identified in Q10.</t>
         </is>
       </c>
     </row>
@@ -2013,7 +2042,7 @@
       </c>
       <c r="D76" s="5" t="inlineStr">
         <is>
-          <t>Follow-up asked but no specific tradition recorded in transcript.</t>
+          <t>Follow-up asked (Q8) but no specific tradition recorded.</t>
         </is>
       </c>
     </row>
@@ -2499,7 +2528,7 @@
       </c>
       <c r="F2" s="7" t="inlineStr">
         <is>
-          <t>NA</t>
+          <t>low</t>
         </is>
       </c>
       <c r="G2" s="7" t="inlineStr">
@@ -2544,7 +2573,7 @@
       </c>
       <c r="O2" s="7" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>yes</t>
         </is>
       </c>
       <c r="P2" s="7" t="inlineStr">
@@ -2699,7 +2728,7 @@
       </c>
       <c r="AT2" s="7" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>no</t>
         </is>
       </c>
       <c r="AU2" s="7" t="inlineStr">
@@ -2759,7 +2788,7 @@
       </c>
       <c r="BF2" s="7" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>no</t>
         </is>
       </c>
       <c r="BG2" s="7" t="inlineStr">
@@ -2789,12 +2818,12 @@
       </c>
       <c r="BL2" s="7" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>no</t>
         </is>
       </c>
       <c r="BM2" s="7" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>no</t>
         </is>
       </c>
       <c r="BN2" s="7" t="inlineStr">
@@ -3728,4 +3757,128 @@
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B10"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="28" customWidth="1" min="1" max="1"/>
+    <col width="90" customWidth="1" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="8" t="inlineStr">
+        <is>
+          <t>Stakeholder Analysis — NPL_1</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="9" t="inlineStr">
+        <is>
+          <t>Interview ID</t>
+        </is>
+      </c>
+      <c r="B3" s="10" t="inlineStr">
+        <is>
+          <t>NPL_1</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="9" t="inlineStr">
+        <is>
+          <t>Country</t>
+        </is>
+      </c>
+      <c r="B4" s="10" t="inlineStr">
+        <is>
+          <t>NEPAL</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="9" t="inlineStr">
+        <is>
+          <t>Coded actor type</t>
+        </is>
+      </c>
+      <c r="B5" s="10" t="inlineStr">
+        <is>
+          <t>governmental</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="9" t="inlineStr">
+        <is>
+          <t>Likely affiliation</t>
+        </is>
+      </c>
+      <c r="B6" s="10" t="inlineStr">
+        <is>
+          <t>Department of Environment / Ministry of Forests and Environment (federal)</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="9" t="inlineStr">
+        <is>
+          <t>Role in plastic governance</t>
+        </is>
+      </c>
+      <c r="B7" s="10" t="inlineStr">
+        <is>
+          <t>National policy design, monitoring of producers/markets, awareness campaigns, SWM Act revision</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="9" t="inlineStr">
+        <is>
+          <t>Perspective</t>
+        </is>
+      </c>
+      <c r="B8" s="10" t="inlineStr">
+        <is>
+          <t>Insider — describes measures as 'we' (government actor implementing national plastic policy)</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="9" t="inlineStr">
+        <is>
+          <t>Confidence</t>
+        </is>
+      </c>
+      <c r="B9" s="10" t="inlineStr">
+        <is>
+          <t>High for governmental coding; see RSCT note below</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="9" t="inlineStr">
+        <is>
+          <t>RSCT note</t>
+        </is>
+      </c>
+      <c r="B10" s="10" t="inlineStr">
+        <is>
+          <t>Page 1 contains RSCT cooperative profile notes (est. 1991, 200+ cooperatives, grassroots loans, recently urban plastics). This does not match the interview voice in Themes A–D, which is clearly a federal ministry/department official. RSCT notes are treated as misplaced interviewer notes, not the coded stakeholder.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:B1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Verify NPL_1 coding against DoE interview notes
Confirm Environmental Department interview (Deepak Diwali, Deputy
Director, 23 June 2025). Recode from Notes1 primary and Notes2
supplementary sources. Add Sources sheet and updated stakeholder profile.

Co-authored-by: Vaibhav <shivrain@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/interview_coding_NPL_1.xlsx
+++ b/interview_coding_NPL_1.xlsx
@@ -11,6 +11,7 @@
     <sheet name="Wide Format" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="Codebook Reference" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="Stakeholder Analysis" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Sources" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -540,7 +541,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Interview: NPL_1  |  Country: NEPAL  |  Actor: Federal governmental (Department of Environment / Ministry)  |  Source: Interview Guideline — Environmental Department (June 2023)</t>
+          <t>Interview: NPL_1 (no. 5)  |  Country: NEPAL  |  Department of Environment — Deepak Diwali, Deputy Director  |  23 June 2025  |  Verified against Notes1 &amp; Notes2</t>
         </is>
       </c>
     </row>
@@ -638,7 +639,7 @@
       </c>
       <c r="D8" s="5" t="inlineStr">
         <is>
-          <t>Federal governmental actor (Department of Environment). Uses first-person 'we' for policy implementation, ministry-only questions (4.a/4.b), and describes Chief Secretary committee oversight.</t>
+          <t>Deepak Diwali, Deputy Director (Pollution Control — air and plastics), Department of Environment. Interview no. 5, 23 June 2025.</t>
         </is>
       </c>
     </row>
@@ -660,7 +661,7 @@
       </c>
       <c r="D9" s="4" t="inlineStr">
         <is>
-          <t>Public is ignorant; people know plastic is a problem but not the full extent.</t>
+          <t>Notes1 Q10: public needs awareness on health impacts; behavioural/mindset change needed. Notes2: people know but not the full extent.</t>
         </is>
       </c>
     </row>
@@ -682,7 +683,7 @@
       </c>
       <c r="D10" s="5" t="inlineStr">
         <is>
-          <t>Low political priority among decision-makers: 'no political will', plastics/waste 'not a priority' and 'stops at major' level.</t>
+          <t>Notes2: no political will; plastics/waste not a priority at decision-maker level.</t>
         </is>
       </c>
     </row>
@@ -704,7 +705,7 @@
       </c>
       <c r="D11" s="4" t="inlineStr">
         <is>
-          <t>Serious issue across rivers, lakes, land, forests; microplastics in Himalayan snow.</t>
+          <t>Notes1: problem everywhere; rivers; high leakage in water bodies; microplastics pollution.</t>
         </is>
       </c>
     </row>
@@ -726,7 +727,7 @@
       </c>
       <c r="D12" s="5" t="inlineStr">
         <is>
-          <t>Blocking sewer systems; leakage into waterways; landfill pressure.</t>
+          <t>Notes2: landfills full, blocking sewer systems. Notes1: leakage into water bodies.</t>
         </is>
       </c>
     </row>
@@ -748,7 +749,7 @@
       </c>
       <c r="D13" s="4" t="inlineStr">
         <is>
-          <t>Lots of plastics are produced.</t>
+          <t>Notes2: lots of plastics produced.</t>
         </is>
       </c>
     </row>
@@ -770,7 +771,7 @@
       </c>
       <c r="D14" s="5" t="inlineStr">
         <is>
-          <t>Inadequate waste management; limited economically viable recycling for single-use items.</t>
+          <t>Notes1: single-use plastics not economically viable to recycle; MRFs to recycling units.</t>
         </is>
       </c>
     </row>
@@ -792,7 +793,7 @@
       </c>
       <c r="D15" s="4" t="inlineStr">
         <is>
-          <t>Waste management for plastics is inadequate.</t>
+          <t>Notes1: lack of plastic waste management; high leakage in water bodies.</t>
         </is>
       </c>
     </row>
@@ -814,7 +815,7 @@
       </c>
       <c r="D16" s="5" t="inlineStr">
         <is>
-          <t>High production rates mentioned.</t>
+          <t>Notes2: high production rates.</t>
         </is>
       </c>
     </row>
@@ -836,7 +837,7 @@
       </c>
       <c r="D17" s="4" t="inlineStr">
         <is>
-          <t>Biodegradable alternatives limited and costly (~100 NPR/kg more).</t>
+          <t>Notes1: non-availability of alternative options; biodegradable plastics costly.</t>
         </is>
       </c>
     </row>
@@ -848,7 +849,7 @@
       </c>
       <c r="B18" s="5" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>yes</t>
         </is>
       </c>
       <c r="C18" s="5" t="inlineStr">
@@ -856,7 +857,11 @@
           <t>Lack of segregation was mentioned: yes/no</t>
         </is>
       </c>
-      <c r="D18" s="5" t="inlineStr"/>
+      <c r="D18" s="5" t="inlineStr">
+        <is>
+          <t>Notes1 Q10: need for separate collection and segregation of plastics implied as gap.</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="4" t="inlineStr">
@@ -876,7 +881,7 @@
       </c>
       <c r="D19" s="4" t="inlineStr">
         <is>
-          <t>Import is part of the problem space: ban on production, import, and use of bags under 40 microns explicitly targets imported plastics.</t>
+          <t>Notes1: restriction on import and use of plastic less than 40 microns in place.</t>
         </is>
       </c>
     </row>
@@ -888,7 +893,7 @@
       </c>
       <c r="B20" s="5" t="inlineStr">
         <is>
-          <t>water, cities, biodiversity, health, agriculture</t>
+          <t>water, health</t>
         </is>
       </c>
       <c r="C20" s="5" t="inlineStr">
@@ -898,7 +903,7 @@
       </c>
       <c r="D20" s="5" t="inlineStr">
         <is>
-          <t>Water (rivers/lakes), cities (sewers/urban), biodiversity (forests), health (burning/indoor air), agriculture (research gap noted for Chitwan).</t>
+          <t>Notes1: rivers/water bodies, microplastics. Notes1 Q10: health impacts. Notes2: burning/indoor health, agriculture research gap (Chitwan).</t>
         </is>
       </c>
     </row>
@@ -956,7 +961,7 @@
       </c>
       <c r="D23" s="4" t="inlineStr">
         <is>
-          <t>Stakeholders are not collaborating or coordinating.</t>
+          <t>Notes2: stakeholders not collaborating or coordinating.</t>
         </is>
       </c>
     </row>
@@ -978,7 +983,7 @@
       </c>
       <c r="D24" s="5" t="inlineStr">
         <is>
-          <t>Challenges differ across national, district, and municipal levels; SWM Act revision needed for federal governance alignment.</t>
+          <t>Notes1 Q10: central govt policy vs LG implementation; municipals manage landfills, DoE monitors markets — multi-level split.</t>
         </is>
       </c>
     </row>
@@ -990,7 +995,7 @@
       </c>
       <c r="B25" s="4" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>yes</t>
         </is>
       </c>
       <c r="C25" s="4" t="inlineStr">
@@ -998,7 +1003,11 @@
           <t>Unclear responsibilities among the involved actors</t>
         </is>
       </c>
-      <c r="D25" s="4" t="inlineStr"/>
+      <c r="D25" s="4" t="inlineStr">
+        <is>
+          <t>Notes1 Q5: LG responsible on ground but DoE role questioned; municipals manage landfills but DoE does not monitor them.</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="5" t="inlineStr">
@@ -1036,7 +1045,7 @@
       </c>
       <c r="D27" s="4" t="inlineStr">
         <is>
-          <t>Department of Environment, Chief Secretary committee, Department of Commerce and Supplies.</t>
+          <t>Department of Environment, Department of Commerce and Supplies, central government policy.</t>
         </is>
       </c>
     </row>
@@ -1076,7 +1085,7 @@
       </c>
       <c r="D29" s="4" t="inlineStr">
         <is>
-          <t>Local governments lead waste management and collection.</t>
+          <t>Notes1: LG responsible on ground; municipals manage landfills; LG monitors markets.</t>
         </is>
       </c>
     </row>
@@ -1116,7 +1125,7 @@
       </c>
       <c r="D31" s="4" t="inlineStr">
         <is>
-          <t>Private companies and contractors in collection/recycling.</t>
+          <t>Notes1: recycling industry; formally established industries monitored.</t>
         </is>
       </c>
     </row>
@@ -1128,7 +1137,7 @@
       </c>
       <c r="B32" s="5" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>no</t>
         </is>
       </c>
       <c r="C32" s="5" t="inlineStr">
@@ -1136,11 +1145,7 @@
           <t>Mentioned: yes/no</t>
         </is>
       </c>
-      <c r="D32" s="5" t="inlineStr">
-        <is>
-          <t>NGOs operate recovery facilities and awareness campaigns.</t>
-        </is>
-      </c>
+      <c r="D32" s="5" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" s="4" t="inlineStr">
@@ -1160,7 +1165,7 @@
       </c>
       <c r="D33" s="4" t="inlineStr">
         <is>
-          <t>Cites studies on microplastics; notes limited research on health/environmental effects.</t>
+          <t>Notes2: not much research on effects of plastics; more research needed.</t>
         </is>
       </c>
     </row>
@@ -1182,7 +1187,7 @@
       </c>
       <c r="D34" s="5" t="inlineStr">
         <is>
-          <t>Household waste reduction discussed; 300 NPR/month collector incentive mentioned (household incentive, not a product tax).</t>
+          <t>Notes1 Q9–10: waste producers; implementation at household level; Notes2: 300 NPR household incentive.</t>
         </is>
       </c>
     </row>
@@ -1194,7 +1199,7 @@
       </c>
       <c r="B35" s="4" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>yes</t>
         </is>
       </c>
       <c r="C35" s="4" t="inlineStr">
@@ -1202,7 +1207,11 @@
           <t>Mentioned: yes/no</t>
         </is>
       </c>
-      <c r="D35" s="4" t="inlineStr"/>
+      <c r="D35" s="4" t="inlineStr">
+        <is>
+          <t>Notes1 Q10: schools mentioned for implementation; kids already taught about plastics.</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="5" t="inlineStr">
@@ -1222,7 +1231,7 @@
       </c>
       <c r="D36" s="5" t="inlineStr">
         <is>
-          <t>Private contractors, plastic producers, and markets monitored by Department of Environment.</t>
+          <t>Notes1: plastic producers monitored; informal industries harder to surveil.</t>
         </is>
       </c>
     </row>
@@ -1262,7 +1271,7 @@
       </c>
       <c r="D38" s="5" t="inlineStr">
         <is>
-          <t>Implementation is always the problem; monitoring cited as barrier.</t>
+          <t>Notes1: lack of surveillance; monitors only 2–3 times/year; too few staff. Notes2: implementation/monitoring is the problem.</t>
         </is>
       </c>
     </row>
@@ -1284,7 +1293,7 @@
       </c>
       <c r="D39" s="4" t="inlineStr">
         <is>
-          <t>Funds exist but are not released; earmarked funds may be frozen if unused.</t>
+          <t>Notes2: funds exist but not released; earmarked funds frozen if unused. Notes1: grant/subsidy provisions being developed for industry shift.</t>
         </is>
       </c>
     </row>
@@ -1306,7 +1315,7 @@
       </c>
       <c r="D40" s="5" t="inlineStr">
         <is>
-          <t>Limited knowledge and research on health/environmental effects.</t>
+          <t>Notes2: not much research/knowledge on plastic effects.</t>
         </is>
       </c>
     </row>
@@ -1328,7 +1337,7 @@
       </c>
       <c r="D41" s="4" t="inlineStr">
         <is>
-          <t>Facilities exist in at least some contexts ('facility is there'); not coded as a primary lack-of-infrastructure barrier.</t>
+          <t>Notes2: facilities exist in some contexts. Notes1: MRFs in use — not coded as primary infrastructure gap.</t>
         </is>
       </c>
     </row>
@@ -1350,7 +1359,7 @@
       </c>
       <c r="D42" s="5" t="inlineStr">
         <is>
-          <t>Weak enforcement; cheaper plastics remain in use despite bans.</t>
+          <t>Notes1: no penalty in place; lack of surveillance. Notes1/2: weak enforcement.</t>
         </is>
       </c>
     </row>
@@ -1408,7 +1417,7 @@
       </c>
       <c r="D45" s="4" t="inlineStr">
         <is>
-          <t>Ban on production, import, and use of plastic bags under 40 microns.</t>
+          <t>Notes1: restriction on import and use of plastic &lt;40 microns.</t>
         </is>
       </c>
     </row>
@@ -1430,7 +1439,7 @@
       </c>
       <c r="D46" s="5" t="inlineStr">
         <is>
-          <t>Government documentaries, traditional/social media, website materials.</t>
+          <t>Notes1 Q10: awareness campaigns and advocacy through documentaries.</t>
         </is>
       </c>
     </row>
@@ -1442,7 +1451,7 @@
       </c>
       <c r="B47" s="4" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>yes</t>
         </is>
       </c>
       <c r="C47" s="4" t="inlineStr">
@@ -1450,7 +1459,11 @@
           <t>Education programs</t>
         </is>
       </c>
-      <c r="D47" s="4" t="inlineStr"/>
+      <c r="D47" s="4" t="inlineStr">
+        <is>
+          <t>Notes1 Q10: education in schools; kids taught about plastics.</t>
+        </is>
+      </c>
     </row>
     <row r="48">
       <c r="A48" s="5" t="inlineStr">
@@ -1506,7 +1519,7 @@
       </c>
       <c r="D50" s="5" t="inlineStr">
         <is>
-          <t>No levy/tax on specific products coded. The 300 NPR/month measure is a household waste-reduction incentive for collectors, not a bag tax/levy.</t>
+          <t>No product levy/tax coded. Notes1: planned grant/subsidy for industry shift (financial incentive, not a bag tax).</t>
         </is>
       </c>
     </row>
@@ -1528,7 +1541,7 @@
       </c>
       <c r="D51" s="4" t="inlineStr">
         <is>
-          <t>Ban on bags under 40 microns and plastic decorative flowers.</t>
+          <t>Notes1: ban on plastic flowers and bags (&lt;40 microns).</t>
         </is>
       </c>
     </row>
@@ -1550,7 +1563,7 @@
       </c>
       <c r="D52" s="5" t="inlineStr">
         <is>
-          <t>Biodegradable starch bags discussed as existing but costly alternative.</t>
+          <t>Notes1: biodegradable plastics produced; govt exploring subsidies for environment-friendly alternatives.</t>
         </is>
       </c>
     </row>
@@ -1608,7 +1621,7 @@
       </c>
       <c r="D55" s="4" t="inlineStr">
         <is>
-          <t>Material recovery facilities send recyclables to processing units.</t>
+          <t>Notes1: MRFs and recycling units; circular economy discussed.</t>
         </is>
       </c>
     </row>
@@ -1630,7 +1643,7 @@
       </c>
       <c r="D56" s="5" t="inlineStr">
         <is>
-          <t>Collection by local governments or private contractors.</t>
+          <t>Notes1 Q10: collection system with separate collection needed/implied as measure.</t>
         </is>
       </c>
     </row>
@@ -1670,7 +1683,7 @@
       </c>
       <c r="D58" s="5" t="inlineStr">
         <is>
-          <t>High-level committee chaired by Chief Secretary oversees measures.</t>
+          <t>Notes1: need for a specific plastics management guideline (national framework).</t>
         </is>
       </c>
     </row>
@@ -1692,7 +1705,7 @@
       </c>
       <c r="D59" s="4" t="inlineStr">
         <is>
-          <t>EPR framed as key missing responsibility mechanism.</t>
+          <t>Notes1: EPR / polluters-pay principle; clarify DoE monitoring role.</t>
         </is>
       </c>
     </row>
@@ -1714,7 +1727,7 @@
       </c>
       <c r="D60" s="5" t="inlineStr">
         <is>
-          <t>EPR identified as key gap; no producer responsibility in Nepal.</t>
+          <t>Notes1: no EPR in Nepal; polluters-pay principle recommended.</t>
         </is>
       </c>
     </row>
@@ -1736,7 +1749,7 @@
       </c>
       <c r="D61" s="4" t="inlineStr">
         <is>
-          <t>Need for communication and awareness on how to act.</t>
+          <t>Notes1 Q10: awareness on health impacts; behavioural/mindset change needed.</t>
         </is>
       </c>
     </row>
@@ -1748,7 +1761,7 @@
       </c>
       <c r="B62" s="5" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>yes</t>
         </is>
       </c>
       <c r="C62" s="5" t="inlineStr">
@@ -1758,7 +1771,7 @@
       </c>
       <c r="D62" s="5" t="inlineStr">
         <is>
-          <t>Collection/recycling encouraged, but segregation not proposed as a forward solution.</t>
+          <t>Notes1 Theme D &amp; Q10: segregation of plastics; separate collection; systematic circulation/circular economy.</t>
         </is>
       </c>
     </row>
@@ -1796,7 +1809,11 @@
           <t>New raw materials</t>
         </is>
       </c>
-      <c r="D64" s="5" t="inlineStr"/>
+      <c r="D64" s="5" t="inlineStr">
+        <is>
+          <t>Notes1: circular economy; MRFs to recycling units.</t>
+        </is>
+      </c>
     </row>
     <row r="65">
       <c r="A65" s="4" t="inlineStr">
@@ -1814,7 +1831,11 @@
           <t>Education programs at schools</t>
         </is>
       </c>
-      <c r="D65" s="4" t="inlineStr"/>
+      <c r="D65" s="4" t="inlineStr">
+        <is>
+          <t>Notes1 Q9–10: education for plastic producers; schools; public learning on health impacts.</t>
+        </is>
+      </c>
     </row>
     <row r="66">
       <c r="A66" s="5" t="inlineStr">
@@ -1824,7 +1845,7 @@
       </c>
       <c r="B66" s="5" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>yes</t>
         </is>
       </c>
       <c r="C66" s="5" t="inlineStr">
@@ -1832,7 +1853,11 @@
           <t>Capacity-building programs</t>
         </is>
       </c>
-      <c r="D66" s="5" t="inlineStr"/>
+      <c r="D66" s="5" t="inlineStr">
+        <is>
+          <t>Notes1: inadequate monitoring due to too few staff (only 2–3 inspections/year).</t>
+        </is>
+      </c>
     </row>
     <row r="67">
       <c r="A67" s="4" t="inlineStr">
@@ -1852,7 +1877,7 @@
       </c>
       <c r="D67" s="4" t="inlineStr">
         <is>
-          <t>R&amp;D needed for affordable alternatives.</t>
+          <t>Notes2: R&amp;D for alternatives needed. Notes1: need environment-friendly plastics.</t>
         </is>
       </c>
     </row>
@@ -1890,11 +1915,7 @@
           <t>Ban of products</t>
         </is>
       </c>
-      <c r="D69" s="4" t="inlineStr">
-        <is>
-          <t>Bans described as existing policy; forward-looking solutions emphasize EPR, R&amp;D, communication, and mitigation/adaptation rather than new bans.</t>
-        </is>
-      </c>
+      <c r="D69" s="4" t="inlineStr"/>
     </row>
     <row r="70">
       <c r="A70" s="5" t="inlineStr">
@@ -1914,7 +1935,7 @@
       </c>
       <c r="D70" s="5" t="inlineStr">
         <is>
-          <t>Financial support identified in Q10.</t>
+          <t>Notes1: incentives for alternatives; planned grants to shift industry from 40-micron plastics.</t>
         </is>
       </c>
     </row>
@@ -1936,7 +1957,7 @@
       </c>
       <c r="D71" s="4" t="inlineStr">
         <is>
-          <t>Infrastructural support identified in Q10.</t>
+          <t>Notes1 Q10: collection system, separate collection, biodegradable waste to manure.</t>
         </is>
       </c>
     </row>
@@ -1958,7 +1979,7 @@
       </c>
       <c r="D72" s="5" t="inlineStr">
         <is>
-          <t>Affordable eco-friendly substitutes needed before behaviour change.</t>
+          <t>Notes1: need affordable eco-friendly alternatives; subsidy for biodegradable products.</t>
         </is>
       </c>
     </row>
@@ -1998,7 +2019,7 @@
       </c>
       <c r="D74" s="5" t="inlineStr">
         <is>
-          <t>Enforcement procedures needed alongside bans.</t>
+          <t>Notes1: no penalty in place; need stronger enforcement.</t>
         </is>
       </c>
     </row>
@@ -2020,7 +2041,7 @@
       </c>
       <c r="D75" s="4" t="inlineStr">
         <is>
-          <t>Monitoring improvements implied from implementation challenges.</t>
+          <t>Notes1: strengthen DoE monitoring; increase frequency beyond 2–3 times/year.</t>
         </is>
       </c>
     </row>
@@ -2042,7 +2063,7 @@
       </c>
       <c r="D76" s="5" t="inlineStr">
         <is>
-          <t>Follow-up asked (Q8) but no specific tradition recorded.</t>
+          <t>Notes2 follow-up asked; Notes1 cites Bhaktapur as example only — no tradition coded.</t>
         </is>
       </c>
     </row>
@@ -2568,234 +2589,234 @@
       </c>
       <c r="N2" s="7" t="inlineStr">
         <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="O2" s="7" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="P2" s="7" t="inlineStr">
+        <is>
+          <t>water, health</t>
+        </is>
+      </c>
+      <c r="Q2" s="7" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="R2" s="7" t="inlineStr">
+        <is>
           <t>no</t>
         </is>
       </c>
-      <c r="O2" s="7" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="P2" s="7" t="inlineStr">
-        <is>
-          <t>water, cities, biodiversity, health, agriculture</t>
-        </is>
-      </c>
-      <c r="Q2" s="7" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="R2" s="7" t="inlineStr">
+      <c r="S2" s="7" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="T2" s="7" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="U2" s="7" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="V2" s="7" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="W2" s="7" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="X2" s="7" t="inlineStr">
         <is>
           <t>no</t>
         </is>
       </c>
-      <c r="S2" s="7" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="T2" s="7" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="U2" s="7" t="inlineStr">
+      <c r="Y2" s="7" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="Z2" s="7" t="inlineStr">
         <is>
           <t>no</t>
         </is>
       </c>
-      <c r="V2" s="7" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="W2" s="7" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="X2" s="7" t="inlineStr">
+      <c r="AA2" s="7" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="AB2" s="7" t="inlineStr">
         <is>
           <t>no</t>
         </is>
       </c>
-      <c r="Y2" s="7" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="Z2" s="7" t="inlineStr">
+      <c r="AC2" s="7" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="AD2" s="7" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="AE2" s="7" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="AF2" s="7" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="AG2" s="7" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="AH2" s="7" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="AI2" s="7" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="AJ2" s="7" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="AK2" s="7" t="inlineStr">
         <is>
           <t>no</t>
         </is>
       </c>
-      <c r="AA2" s="7" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="AB2" s="7" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="AC2" s="7" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="AD2" s="7" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="AE2" s="7" t="inlineStr">
+      <c r="AL2" s="7" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="AM2" s="7" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="AN2" s="7" t="inlineStr">
         <is>
           <t>no</t>
         </is>
       </c>
-      <c r="AF2" s="7" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="AG2" s="7" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="AH2" s="7" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="AI2" s="7" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="AJ2" s="7" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="AK2" s="7" t="inlineStr">
+      <c r="AO2" s="7" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="AP2" s="7" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="AQ2" s="7" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="AR2" s="7" t="inlineStr">
         <is>
           <t>no</t>
         </is>
       </c>
-      <c r="AL2" s="7" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="AM2" s="7" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="AN2" s="7" t="inlineStr">
+      <c r="AS2" s="7" t="inlineStr">
         <is>
           <t>no</t>
         </is>
       </c>
-      <c r="AO2" s="7" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="AP2" s="7" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="AQ2" s="7" t="inlineStr">
+      <c r="AT2" s="7" t="inlineStr">
         <is>
           <t>no</t>
         </is>
       </c>
-      <c r="AR2" s="7" t="inlineStr">
+      <c r="AU2" s="7" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="AV2" s="7" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="AW2" s="7" t="inlineStr">
         <is>
           <t>no</t>
         </is>
       </c>
-      <c r="AS2" s="7" t="inlineStr">
+      <c r="AX2" s="7" t="inlineStr">
         <is>
           <t>no</t>
         </is>
       </c>
-      <c r="AT2" s="7" t="inlineStr">
+      <c r="AY2" s="7" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="AZ2" s="7" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="BA2" s="7" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="BB2" s="7" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="BC2" s="7" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="BD2" s="7" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="BE2" s="7" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="BF2" s="7" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="BG2" s="7" t="inlineStr">
         <is>
           <t>no</t>
         </is>
       </c>
-      <c r="AU2" s="7" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="AV2" s="7" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="AW2" s="7" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="AX2" s="7" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="AY2" s="7" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="AZ2" s="7" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="BA2" s="7" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="BB2" s="7" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="BC2" s="7" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="BD2" s="7" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="BE2" s="7" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="BF2" s="7" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="BG2" s="7" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
       <c r="BH2" s="7" t="inlineStr">
         <is>
           <t>yes</t>
@@ -2808,7 +2829,7 @@
       </c>
       <c r="BJ2" s="7" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>yes</t>
         </is>
       </c>
       <c r="BK2" s="7" t="inlineStr">
@@ -3765,7 +3786,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B10"/>
+  <dimension ref="A1:B13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -3806,72 +3827,172 @@
     <row r="5">
       <c r="A5" s="9" t="inlineStr">
         <is>
-          <t>Coded actor type</t>
+          <t>Interview number</t>
         </is>
       </c>
       <c r="B5" s="10" t="inlineStr">
         <is>
-          <t>governmental</t>
+          <t>5</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="9" t="inlineStr">
         <is>
-          <t>Likely affiliation</t>
+          <t>Interview date</t>
         </is>
       </c>
       <c r="B6" s="10" t="inlineStr">
         <is>
-          <t>Department of Environment / Ministry of Forests and Environment (federal)</t>
+          <t>23 June 2025 (3:50pm – 4:40pm)</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="9" t="inlineStr">
         <is>
-          <t>Role in plastic governance</t>
+          <t>Affiliation</t>
         </is>
       </c>
       <c r="B7" s="10" t="inlineStr">
         <is>
-          <t>National policy design, monitoring of producers/markets, awareness campaigns, SWM Act revision</t>
+          <t>Department of Environment, Ministry of Forests and Environment</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="9" t="inlineStr">
         <is>
-          <t>Perspective</t>
+          <t>Interviewee</t>
         </is>
       </c>
       <c r="B8" s="10" t="inlineStr">
         <is>
-          <t>Insider — describes measures as 'we' (government actor implementing national plastic policy)</t>
+          <t>Deepak Diwali — Deputy Director, Pollution Control (air and plastics)</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="9" t="inlineStr">
         <is>
-          <t>Confidence</t>
+          <t>Coded actor type</t>
         </is>
       </c>
       <c r="B9" s="10" t="inlineStr">
         <is>
-          <t>High for governmental coding; see RSCT note below</t>
+          <t>governmental</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="9" t="inlineStr">
         <is>
-          <t>RSCT note</t>
+          <t>Role in plastic governance</t>
         </is>
       </c>
       <c r="B10" s="10" t="inlineStr">
         <is>
-          <t>Page 1 contains RSCT cooperative profile notes (est. 1991, 200+ cooperatives, grassroots loans, recently urban plastics). This does not match the interview voice in Themes A–D, which is clearly a federal ministry/department official. RSCT notes are treated as misplaced interviewer notes, not the coded stakeholder.</t>
+          <t>Federal monitoring of plastic producers/markets; policy instruments (import restrictions, bans); SWM Act revision; coordination with local governments and Department of Commerce and Supplies</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="9" t="inlineStr">
+        <is>
+          <t>Perspective</t>
+        </is>
+      </c>
+      <c r="B11" s="10" t="inlineStr">
+        <is>
+          <t>Insider — describes DoE monitoring role, planned grants, and national policy instruments</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="9" t="inlineStr">
+        <is>
+          <t>Verification status</t>
+        </is>
+      </c>
+      <c r="B12" s="10" t="inlineStr">
+        <is>
+          <t>Confirmed Environmental Department / Ministry interview</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="9" t="inlineStr">
+        <is>
+          <t>Source documents</t>
+        </is>
+      </c>
+      <c r="B13" s="10" t="inlineStr">
+        <is>
+          <t>Notes1 (primary), Notes2 (supplementary)</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:B1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B5"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="42" customWidth="1" min="1" max="1"/>
+    <col width="60" customWidth="1" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="8" t="inlineStr">
+        <is>
+          <t>Source Documents Used for Verification</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="9" t="inlineStr">
+        <is>
+          <t>Notes1 — Department of Environment (primary)</t>
+        </is>
+      </c>
+      <c r="B3" s="10" t="inlineStr">
+        <is>
+          <t>Interview no. 5, 23 June 2025, 3:50–4:40pm</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="9" t="inlineStr">
+        <is>
+          <t>Notes2 — Department of Environment (supplementary)</t>
+        </is>
+      </c>
+      <c r="B4" s="10" t="inlineStr">
+        <is>
+          <t>Interview guideline with interviewer bullet notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="9" t="inlineStr">
+        <is>
+          <t>Codebook</t>
+        </is>
+      </c>
+      <c r="B5" s="10" t="inlineStr">
+        <is>
+          <t>Overview All Interviews — NEW Codebook</t>
         </is>
       </c>
     </row>

</xml_diff>